<commit_message>
Suma conformidad, origen y contexto de cada cliente contado por Mateo
Peque Mundos pasa a trabajo unico (campana de invierno), los 13 trabajos
de la web sin cobro quedan como demo y Medisur como cliente sin cobro.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/comercial/TNR-datos-para-el-analisis.xlsx
+++ b/comercial/TNR-datos-para-el-analisis.xlsx
@@ -743,6 +743,7 @@
     <col width="15" customWidth="1" min="12" max="12"/>
     <col width="16" customWidth="1" min="13" max="13"/>
     <col width="34" customWidth="1" min="14" max="14"/>
+    <col width="24" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -831,6 +832,11 @@
           <t>Notas</t>
         </is>
       </c>
+      <c r="O4" s="6" t="inlineStr">
+        <is>
+          <t>Origen del cliente</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="11" t="inlineStr">
@@ -870,7 +876,11 @@
       <c r="I5" s="12" t="n">
         <v>152000</v>
       </c>
-      <c r="J5" s="11" t="n"/>
+      <c r="J5" s="11" t="inlineStr">
+        <is>
+          <t>Muy conforme (según Mateo)</t>
+        </is>
+      </c>
       <c r="K5" s="11" t="inlineStr">
         <is>
           <t>Real</t>
@@ -884,10 +894,14 @@
       </c>
       <c r="N5" s="11" t="inlineStr">
         <is>
-          <t>Todo cobrado. El cliente que más facturó: 934.000 en 3 meses.</t>
-        </is>
-      </c>
-      <c r="O5" s="13" t="n"/>
+          <t>Agus. Paga a tiempo, nos ve profesionales, entregamos antes de lo prometido. Ads para EE.UU. 120.000/mes + mantenimiento 32.000/mes.</t>
+        </is>
+      </c>
+      <c r="O5" s="13" t="inlineStr">
+        <is>
+          <t>Referido de Thiago</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="14" t="inlineStr">
@@ -931,7 +945,11 @@
       <c r="I6" s="15" t="n">
         <v>90000</v>
       </c>
-      <c r="J6" s="14" t="n"/>
+      <c r="J6" s="14" t="inlineStr">
+        <is>
+          <t>A confirmar</t>
+        </is>
+      </c>
       <c r="K6" s="14" t="inlineStr">
         <is>
           <t>Real</t>
@@ -945,10 +963,14 @@
       </c>
       <c r="N6" s="14" t="inlineStr">
         <is>
-          <t>Único mensual que ya pagó 4 meses seguidos. Falta cargar el cobro de septiembre (el último fue el 22/08).</t>
-        </is>
-      </c>
-      <c r="O6" s="16" t="n"/>
+          <t>4º mes. 90.000 por 2 estáticas + 2 carruseles + 2 reels. Incluye una campaña de anuncios gratis; después una paga de 100.000.</t>
+        </is>
+      </c>
+      <c r="O6" s="16" t="inlineStr">
+        <is>
+          <t>A confirmar</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="14" t="inlineStr">
@@ -992,7 +1014,11 @@
       <c r="I7" s="15" t="n">
         <v>100000</v>
       </c>
-      <c r="J7" s="14" t="n"/>
+      <c r="J7" s="14" t="inlineStr">
+        <is>
+          <t>Muy conforme (según Mateo: "la tenemos clara")</t>
+        </is>
+      </c>
       <c r="K7" s="14" t="inlineStr">
         <is>
           <t>Real</t>
@@ -1006,10 +1032,14 @@
       </c>
       <c r="N7" s="14" t="inlineStr">
         <is>
-          <t>Facturado 450.000, cobrado 400.000: debe 50.000.</t>
-        </is>
-      </c>
-      <c r="O7" s="16" t="n"/>
+          <t>Claudio. Web 350.000 + Google Ads 100.000/mes + mantenimiento web 100.000 (confirmar si es mensual).</t>
+        </is>
+      </c>
+      <c r="O7" s="16" t="inlineStr">
+        <is>
+          <t>A confirmar</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="14" t="inlineStr">
@@ -1049,7 +1079,11 @@
       <c r="I8" s="15" t="n">
         <v>108000</v>
       </c>
-      <c r="J8" s="14" t="n"/>
+      <c r="J8" s="14" t="inlineStr">
+        <is>
+          <t>A confirmar</t>
+        </is>
+      </c>
       <c r="K8" s="14" t="inlineStr">
         <is>
           <t>Real</t>
@@ -1063,10 +1097,14 @@
       </c>
       <c r="N8" s="14" t="inlineStr">
         <is>
-          <t>Primer mes. Todavía no demostró que renueva.</t>
-        </is>
-      </c>
-      <c r="O8" s="16" t="n"/>
+          <t>Paga 120.000 bruto; 12.000 al vendedor (el CRM guarda el neto: 108.000). 16 piezas/mes hechas con Claude, sin estrategia; no hay engagement.</t>
+        </is>
+      </c>
+      <c r="O8" s="16" t="inlineStr">
+        <is>
+          <t>Vendedor (cold call)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="14" t="inlineStr">
@@ -1110,7 +1148,11 @@
       <c r="I9" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="J9" s="14" t="n"/>
+      <c r="J9" s="14" t="inlineStr">
+        <is>
+          <t>A confirmar</t>
+        </is>
+      </c>
       <c r="K9" s="14" t="inlineStr">
         <is>
           <t>Real</t>
@@ -1124,10 +1166,14 @@
       </c>
       <c r="N9" s="14" t="inlineStr">
         <is>
-          <t>Facturado 350.000, cobrado 250.000: debe 100.000.</t>
-        </is>
-      </c>
-      <c r="O9" s="16" t="n"/>
+          <t>E-commerce + branding 350.000 a 50.000 por semana (5ª semana). Queremos venderle redes.</t>
+        </is>
+      </c>
+      <c r="O9" s="16" t="inlineStr">
+        <is>
+          <t>A confirmar</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
@@ -1167,7 +1213,11 @@
       <c r="I10" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="J10" s="14" t="n"/>
+      <c r="J10" s="14" t="inlineStr">
+        <is>
+          <t>A confirmar</t>
+        </is>
+      </c>
       <c r="K10" s="14" t="inlineStr">
         <is>
           <t>Real</t>
@@ -1181,10 +1231,14 @@
       </c>
       <c r="N10" s="14" t="inlineStr">
         <is>
-          <t>Facturado 210.000 "con comisión Rega", cobrado 140.000: debe 70.000.</t>
-        </is>
-      </c>
-      <c r="O10" s="16" t="n"/>
+          <t>Web 300.000 bruto; 30% al vendedor (el CRM guarda el neto: 210.000). Pagó 200.000, última cuota de 100.000 el 08/10. Panel nuevo a cobrar: 300.000.</t>
+        </is>
+      </c>
+      <c r="O10" s="16" t="inlineStr">
+        <is>
+          <t>Vendedor (cold call)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="14" t="inlineStr">
@@ -1228,7 +1282,11 @@
       <c r="I11" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="J11" s="14" t="n"/>
+      <c r="J11" s="14" t="inlineStr">
+        <is>
+          <t>A confirmar</t>
+        </is>
+      </c>
       <c r="K11" s="14" t="inlineStr">
         <is>
           <t>Real</t>
@@ -1242,10 +1300,14 @@
       </c>
       <c r="N11" s="14" t="inlineStr">
         <is>
-          <t>Vino de la prospección (respondió el 26/07). Tiene un plan de redes a $0 cargado: trabajo mensual regalado.</t>
-        </is>
-      </c>
-      <c r="O11" s="16" t="n"/>
+          <t>Demo gratis + web 200.000 + 1 mes de redes gratis (está por arrancar). Queremos cerrarle redes pagas por semana.</t>
+        </is>
+      </c>
+      <c r="O11" s="16" t="inlineStr">
+        <is>
+          <t>Prospección por WhatsApp</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
@@ -1289,7 +1351,11 @@
       <c r="I12" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="J12" s="14" t="n"/>
+      <c r="J12" s="14" t="inlineStr">
+        <is>
+          <t>Buena (según Mateo: "nos cayó bien")</t>
+        </is>
+      </c>
       <c r="K12" s="14" t="inlineStr">
         <is>
           <t>Real</t>
@@ -1303,10 +1369,14 @@
       </c>
       <c r="N12" s="14" t="inlineStr">
         <is>
-          <t>Seña de 100.000 sobre 300.000: debe 200.000. Vino de la prospección (demo enviada el 23/07).</t>
-        </is>
-      </c>
-      <c r="O12" s="16" t="n"/>
+          <t>Web 300.000 en 3 cuotas de 100.000; la primera se pagó el 18/09.</t>
+        </is>
+      </c>
+      <c r="O12" s="16" t="inlineStr">
+        <is>
+          <t>Prospección por WhatsApp</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="14" t="inlineStr">
@@ -1350,7 +1420,11 @@
       <c r="I13" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="J13" s="14" t="n"/>
+      <c r="J13" s="14" t="inlineStr">
+        <is>
+          <t>A confirmar</t>
+        </is>
+      </c>
       <c r="K13" s="14" t="inlineStr">
         <is>
           <t>Real</t>
@@ -1364,10 +1438,14 @@
       </c>
       <c r="N13" s="14" t="inlineStr">
         <is>
-          <t>Sin movimiento en el CRM desde junio. Es el contador al que queremos consultar.</t>
-        </is>
-      </c>
-      <c r="O13" s="16" t="n"/>
+          <t>Landing + SEO 150.000. No compró redes (el marido no quería). Hay que recontactar.</t>
+        </is>
+      </c>
+      <c r="O13" s="16" t="inlineStr">
+        <is>
+          <t>Cold call (Mateo)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="14" t="inlineStr">
@@ -1407,7 +1485,11 @@
       <c r="I14" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="J14" s="14" t="n"/>
+      <c r="J14" s="14" t="inlineStr">
+        <is>
+          <t>Mala: nos despidió</t>
+        </is>
+      </c>
       <c r="K14" s="14" t="inlineStr">
         <is>
           <t>Real</t>
@@ -1421,10 +1503,14 @@
       </c>
       <c r="N14" s="14" t="inlineStr">
         <is>
-          <t>Pagó un mes y quedó Inactivo.</t>
-        </is>
-      </c>
-      <c r="O14" s="16" t="n"/>
+          <t>Nos despidió por impuntualidad y contenidos mal publicados. Igual nos trajo a Setup, Peque Mundos y Medisur. Hoy estudia afuera. Mantener la relación.</t>
+        </is>
+      </c>
+      <c r="O14" s="16" t="inlineStr">
+        <is>
+          <t>A confirmar</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="14" t="inlineStr">
@@ -1468,7 +1554,11 @@
       <c r="I15" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="J15" s="14" t="n"/>
+      <c r="J15" s="14" t="inlineStr">
+        <is>
+          <t>A confirmar</t>
+        </is>
+      </c>
       <c r="K15" s="14" t="inlineStr">
         <is>
           <t>Real</t>
@@ -1482,10 +1572,14 @@
       </c>
       <c r="N15" s="14" t="inlineStr">
         <is>
-          <t>Lo vendió Thiago con 10% de descuento. Pagó un mes y quedó Inactivo.</t>
-        </is>
-      </c>
-      <c r="O15" s="16" t="n"/>
+          <t>Trabajo de UNA vez por decisión de la clienta: campaña de vacaciones de invierno. No fue una baja.</t>
+        </is>
+      </c>
+      <c r="O15" s="16" t="inlineStr">
+        <is>
+          <t>Referido de Thiago</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="14" t="inlineStr">
@@ -1529,7 +1623,11 @@
       <c r="I16" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="J16" s="14" t="n"/>
+      <c r="J16" s="14" t="inlineStr">
+        <is>
+          <t>Mala: no paga ni contesta</t>
+        </is>
+      </c>
       <c r="K16" s="14" t="inlineStr">
         <is>
           <t>Real</t>
@@ -1543,10 +1641,14 @@
       </c>
       <c r="N16" s="14" t="inlineStr">
         <is>
-          <t>El CRM dice "Volver a tenerlo". Facturado 360.000, cobrado 205.000: figura una deuda de 155.000 desde junio (puede ser error de carga).</t>
-        </is>
-      </c>
-      <c r="O16" s="16" t="n"/>
+          <t>Segundo cliente. Nos debe 155.000 y no contesta. Contenidos flojos (éramos principiantes). Queremos volver en vacaciones.</t>
+        </is>
+      </c>
+      <c r="O16" s="16" t="inlineStr">
+        <is>
+          <t>A confirmar</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="14" t="inlineStr">
@@ -1590,7 +1692,11 @@
       <c r="I17" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="J17" s="14" t="n"/>
+      <c r="J17" s="14" t="inlineStr">
+        <is>
+          <t>A confirmar</t>
+        </is>
+      </c>
       <c r="K17" s="14" t="inlineStr">
         <is>
           <t>Real</t>
@@ -1604,10 +1710,14 @@
       </c>
       <c r="N17" s="14" t="inlineStr">
         <is>
-          <t>Pagó 360.000 en junio. Inactivo.</t>
-        </is>
-      </c>
-      <c r="O17" s="16" t="n"/>
+          <t>Dos meses de redes + una campaña de anuncios gratis. No entendían lo que se hacía.</t>
+        </is>
+      </c>
+      <c r="O17" s="16" t="inlineStr">
+        <is>
+          <t>Conocidos (profes de fútbol de Mateo)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="14" t="inlineStr">
@@ -1643,7 +1753,11 @@
       <c r="I18" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="J18" s="14" t="n"/>
+      <c r="J18" s="14" t="inlineStr">
+        <is>
+          <t>A confirmar</t>
+        </is>
+      </c>
       <c r="K18" s="14" t="inlineStr">
         <is>
           <t>Real</t>
@@ -1657,10 +1771,14 @@
       </c>
       <c r="N18" s="14" t="inlineStr">
         <is>
-          <t>Pago migrado del registro anterior.</t>
-        </is>
-      </c>
-      <c r="O18" s="16" t="n"/>
+          <t>El primero, principios de febrero. 4 reels a 60.000 cada uno. Hoy trabaja con otra agencia.</t>
+        </is>
+      </c>
+      <c r="O18" s="16" t="inlineStr">
+        <is>
+          <t>A confirmar</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="17" t="inlineStr">
@@ -1679,14 +1797,14 @@
       <c r="J19" s="17" t="n"/>
       <c r="K19" s="17" t="inlineStr">
         <is>
-          <t>A confirmar</t>
+          <t>Demo / no pagó</t>
         </is>
       </c>
       <c r="L19" s="17" t="n"/>
       <c r="M19" s="17" t="n"/>
       <c r="N19" s="17" t="inlineStr">
         <is>
-          <t>Publicado en /trabajos pero NO figura en los clientes del CRM. ¿Pagó? ¿Cuándo y cuánto? Si fue antes de junio, el CRM no lo tiene.</t>
+          <t>Publicado en /trabajos. Según Mateo, los que pagaron están todos en Clientes: este no pagó.</t>
         </is>
       </c>
       <c r="O19" s="16" t="n"/>
@@ -1708,17 +1826,21 @@
       <c r="J20" s="17" t="n"/>
       <c r="K20" s="17" t="inlineStr">
         <is>
-          <t>A confirmar</t>
+          <t>Cliente sin cobro todavía</t>
         </is>
       </c>
       <c r="L20" s="17" t="n"/>
       <c r="M20" s="17" t="n"/>
       <c r="N20" s="17" t="inlineStr">
         <is>
-          <t>Publicado en /trabajos pero NO figura en los clientes del CRM. ¿Pagó? ¿Cuándo y cuánto? Si fue antes de junio, el CRM no lo tiene.</t>
-        </is>
-      </c>
-      <c r="O20" s="16" t="n"/>
+          <t>Lo vendió Thiago. Vemos la ganancia en febrero de 2027. Hasta entonces no entró plata.</t>
+        </is>
+      </c>
+      <c r="O20" s="16" t="inlineStr">
+        <is>
+          <t>Referido de Thiago</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="17" t="inlineStr">
@@ -1737,14 +1859,14 @@
       <c r="J21" s="17" t="n"/>
       <c r="K21" s="17" t="inlineStr">
         <is>
-          <t>A confirmar</t>
+          <t>Demo / no pagó</t>
         </is>
       </c>
       <c r="L21" s="17" t="n"/>
       <c r="M21" s="17" t="n"/>
       <c r="N21" s="17" t="inlineStr">
         <is>
-          <t>Publicado en /trabajos pero NO figura en los clientes del CRM. ¿Pagó? ¿Cuándo y cuánto? Si fue antes de junio, el CRM no lo tiene.</t>
+          <t>Publicado en /trabajos. Según Mateo, los que pagaron están todos en Clientes: este no pagó.</t>
         </is>
       </c>
       <c r="O21" s="16" t="n"/>
@@ -1766,14 +1888,14 @@
       <c r="J22" s="17" t="n"/>
       <c r="K22" s="17" t="inlineStr">
         <is>
-          <t>A confirmar</t>
+          <t>Demo / no pagó</t>
         </is>
       </c>
       <c r="L22" s="17" t="n"/>
       <c r="M22" s="17" t="n"/>
       <c r="N22" s="17" t="inlineStr">
         <is>
-          <t>Publicado en /trabajos pero NO figura en los clientes del CRM. ¿Pagó? ¿Cuándo y cuánto? Si fue antes de junio, el CRM no lo tiene.</t>
+          <t>Publicado en /trabajos. Según Mateo, los que pagaron están todos en Clientes: este no pagó.</t>
         </is>
       </c>
       <c r="O22" s="16" t="n"/>
@@ -1795,14 +1917,14 @@
       <c r="J23" s="17" t="n"/>
       <c r="K23" s="17" t="inlineStr">
         <is>
-          <t>A confirmar</t>
+          <t>Demo / no pagó</t>
         </is>
       </c>
       <c r="L23" s="17" t="n"/>
       <c r="M23" s="17" t="n"/>
       <c r="N23" s="17" t="inlineStr">
         <is>
-          <t>Publicado en /trabajos pero NO figura en los clientes del CRM. ¿Pagó? ¿Cuándo y cuánto? Si fue antes de junio, el CRM no lo tiene.</t>
+          <t>Publicado en /trabajos. Según Mateo, los que pagaron están todos en Clientes: este no pagó.</t>
         </is>
       </c>
       <c r="O23" s="16" t="n"/>
@@ -1824,14 +1946,14 @@
       <c r="J24" s="17" t="n"/>
       <c r="K24" s="17" t="inlineStr">
         <is>
-          <t>A confirmar</t>
+          <t>Demo / no pagó</t>
         </is>
       </c>
       <c r="L24" s="17" t="n"/>
       <c r="M24" s="17" t="n"/>
       <c r="N24" s="17" t="inlineStr">
         <is>
-          <t>Publicado en /trabajos pero NO figura en los clientes del CRM. ¿Pagó? ¿Cuándo y cuánto? Si fue antes de junio, el CRM no lo tiene.</t>
+          <t>Publicado en /trabajos. Según Mateo, los que pagaron están todos en Clientes: este no pagó.</t>
         </is>
       </c>
       <c r="O24" s="16" t="n"/>
@@ -1853,14 +1975,14 @@
       <c r="J25" s="17" t="n"/>
       <c r="K25" s="17" t="inlineStr">
         <is>
-          <t>A confirmar</t>
+          <t>Demo / no pagó</t>
         </is>
       </c>
       <c r="L25" s="17" t="n"/>
       <c r="M25" s="17" t="n"/>
       <c r="N25" s="17" t="inlineStr">
         <is>
-          <t>Publicado en /trabajos pero NO figura en los clientes del CRM. ¿Pagó? ¿Cuándo y cuánto? Si fue antes de junio, el CRM no lo tiene.</t>
+          <t>Publicado en /trabajos. Según Mateo, los que pagaron están todos en Clientes: este no pagó.</t>
         </is>
       </c>
       <c r="O25" s="16" t="n"/>
@@ -1882,14 +2004,14 @@
       <c r="J26" s="17" t="n"/>
       <c r="K26" s="17" t="inlineStr">
         <is>
-          <t>A confirmar</t>
+          <t>Demo / no pagó</t>
         </is>
       </c>
       <c r="L26" s="17" t="n"/>
       <c r="M26" s="17" t="n"/>
       <c r="N26" s="17" t="inlineStr">
         <is>
-          <t>Publicado en /trabajos pero NO figura en los clientes del CRM. ¿Pagó? ¿Cuándo y cuánto? Si fue antes de junio, el CRM no lo tiene.</t>
+          <t>Publicado en /trabajos. Según Mateo, los que pagaron están todos en Clientes: este no pagó.</t>
         </is>
       </c>
       <c r="O26" s="16" t="n"/>
@@ -1911,14 +2033,14 @@
       <c r="J27" s="17" t="n"/>
       <c r="K27" s="17" t="inlineStr">
         <is>
-          <t>A confirmar</t>
+          <t>Demo / no pagó</t>
         </is>
       </c>
       <c r="L27" s="17" t="n"/>
       <c r="M27" s="17" t="n"/>
       <c r="N27" s="17" t="inlineStr">
         <is>
-          <t>Publicado en /trabajos pero NO figura en los clientes del CRM. ¿Pagó? ¿Cuándo y cuánto? Si fue antes de junio, el CRM no lo tiene.</t>
+          <t>Publicado en /trabajos. Según Mateo, los que pagaron están todos en Clientes: este no pagó.</t>
         </is>
       </c>
       <c r="O27" s="16" t="n"/>
@@ -1940,14 +2062,14 @@
       <c r="J28" s="17" t="n"/>
       <c r="K28" s="17" t="inlineStr">
         <is>
-          <t>A confirmar</t>
+          <t>Demo / no pagó</t>
         </is>
       </c>
       <c r="L28" s="17" t="n"/>
       <c r="M28" s="17" t="n"/>
       <c r="N28" s="17" t="inlineStr">
         <is>
-          <t>Publicado en /trabajos pero NO figura en los clientes del CRM. ¿Pagó? ¿Cuándo y cuánto? Si fue antes de junio, el CRM no lo tiene.</t>
+          <t>Publicado en /trabajos. Según Mateo, los que pagaron están todos en Clientes: este no pagó.</t>
         </is>
       </c>
       <c r="O28" s="16" t="n"/>
@@ -1969,14 +2091,14 @@
       <c r="J29" s="17" t="n"/>
       <c r="K29" s="17" t="inlineStr">
         <is>
-          <t>A confirmar</t>
+          <t>Demo / no pagó</t>
         </is>
       </c>
       <c r="L29" s="17" t="n"/>
       <c r="M29" s="17" t="n"/>
       <c r="N29" s="17" t="inlineStr">
         <is>
-          <t>Publicado en /trabajos pero NO figura en los clientes del CRM. ¿Pagó? ¿Cuándo y cuánto? Si fue antes de junio, el CRM no lo tiene.</t>
+          <t>Publicado en /trabajos. Según Mateo, los que pagaron están todos en Clientes: este no pagó.</t>
         </is>
       </c>
       <c r="O29" s="16" t="n"/>
@@ -1998,14 +2120,14 @@
       <c r="J30" s="17" t="n"/>
       <c r="K30" s="17" t="inlineStr">
         <is>
-          <t>A confirmar</t>
+          <t>Demo / no pagó</t>
         </is>
       </c>
       <c r="L30" s="17" t="n"/>
       <c r="M30" s="17" t="n"/>
       <c r="N30" s="17" t="inlineStr">
         <is>
-          <t>Publicado en /trabajos pero NO figura en los clientes del CRM. ¿Pagó? ¿Cuándo y cuánto? Si fue antes de junio, el CRM no lo tiene.</t>
+          <t>Publicado en /trabajos. Según Mateo, los que pagaron están todos en Clientes: este no pagó.</t>
         </is>
       </c>
       <c r="O30" s="16" t="n"/>
@@ -2027,14 +2149,14 @@
       <c r="J31" s="17" t="n"/>
       <c r="K31" s="17" t="inlineStr">
         <is>
-          <t>A confirmar</t>
+          <t>Demo / no pagó</t>
         </is>
       </c>
       <c r="L31" s="17" t="n"/>
       <c r="M31" s="17" t="n"/>
       <c r="N31" s="17" t="inlineStr">
         <is>
-          <t>Publicado en /trabajos pero NO figura en los clientes del CRM. ¿Pagó? ¿Cuándo y cuánto? Si fue antes de junio, el CRM no lo tiene.</t>
+          <t>Publicado en /trabajos. Según Mateo, los que pagaron están todos en Clientes: este no pagó.</t>
         </is>
       </c>
       <c r="O31" s="16" t="n"/>
@@ -2059,7 +2181,7 @@
     <row r="33">
       <c r="A33" s="18" t="inlineStr">
         <is>
-          <t>Las columnas "¿Quedó conforme? 1-5" y "¿Autoriza mostrarlo?" no están en el CRM. Las completan ustedes.</t>
+          <t>Conformidad: está en palabras de ustedes. El número del 1 al 5 lo ponen ustedes.</t>
         </is>
       </c>
       <c r="B33" s="14" t="n"/>
@@ -3229,7 +3351,13 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="6" customHeight="1"/>
+    <row r="3" ht="6" customHeight="1">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Ojo: Ton Cars y Satelital están en NETO (sin la comisión del vendedor). En bruto, septiembre suma 42.000 más.</t>
+        </is>
+      </c>
+    </row>
     <row r="4" ht="34" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
         <is>
@@ -3300,10 +3428,10 @@
         </is>
       </c>
       <c r="B6" s="21" t="n">
-        <v>70000</v>
+        <v>191500</v>
       </c>
       <c r="C6" s="21" t="n">
-        <v>211500</v>
+        <v>90000</v>
       </c>
       <c r="D6" s="21" t="n">
         <v>281500</v>
@@ -3314,7 +3442,7 @@
       <c r="F6" s="20" t="n"/>
       <c r="G6" s="20" t="inlineStr">
         <is>
-          <t>Recurrente: 75% del mes.</t>
+          <t>Recurrente: 32% del mes.</t>
         </is>
       </c>
       <c r="H6" s="16" t="n"/>
@@ -3378,10 +3506,10 @@
         </is>
       </c>
       <c r="B9" s="22" t="n">
-        <v>2520000</v>
+        <v>2641500</v>
       </c>
       <c r="C9" s="22" t="n">
-        <v>1128500</v>
+        <v>1007000</v>
       </c>
       <c r="D9" s="22" t="n">
         <v>3648500</v>
@@ -3392,7 +3520,7 @@
       <c r="F9" s="18" t="n"/>
       <c r="G9" s="18" t="inlineStr">
         <is>
-          <t>Recurrente: 31% de todo lo cobrado desde junio</t>
+          <t>Recurrente: 28% de todo lo cobrado desde junio</t>
         </is>
       </c>
       <c r="H9" s="16" t="n"/>
@@ -3975,7 +4103,6 @@
           <t>Mercado Pago</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -4091,7 +4218,6 @@
           <t>Mercado Pago</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4127,7 +4253,6 @@
           <t>Mercado Pago</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -4163,7 +4288,6 @@
           <t>Efectivo</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -4199,7 +4323,6 @@
           <t>Mercado Pago</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -4217,7 +4340,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Recurrente</t>
+          <t>Proyecto único</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -4237,7 +4360,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Lo vendió Thiago. Cliente hoy Inactivo</t>
+          <t>Campaña de vacaciones de invierno, trabajo único por decisión de la clienta</t>
         </is>
       </c>
     </row>
@@ -4275,7 +4398,6 @@
           <t>Mercado Pago</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -4311,7 +4433,6 @@
           <t>Mercado Pago</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -4347,7 +4468,6 @@
           <t>Transferencia</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -4383,7 +4503,6 @@
           <t>Mercado Pago</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -4499,7 +4618,6 @@
           <t>Mercado Pago</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -4535,7 +4653,6 @@
           <t>Mercado Pago</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -4571,7 +4688,6 @@
           <t>Mercado Pago</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -4607,7 +4723,6 @@
           <t>Efectivo</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -4643,7 +4758,6 @@
           <t>Mercado Pago</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -4679,7 +4793,6 @@
           <t>Mercado Pago</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -4715,7 +4828,6 @@
           <t>Mercado Pago</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -4751,7 +4863,11 @@
           <t>Mercado Pago</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr"/>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Monto neto: sin la comisión del vendedor</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -4787,7 +4903,6 @@
           <t>Mercado Pago</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -4823,7 +4938,6 @@
           <t>Efectivo</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -4859,7 +4973,6 @@
           <t>Efectivo</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -4895,7 +5008,11 @@
           <t>Mercado Pago</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr"/>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Monto neto: sin la comisión del vendedor</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -5011,7 +5128,6 @@
           <t>Mercado Pago</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -5047,7 +5163,6 @@
           <t>Mercado Pago</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Conformidad y origen de F5, MC E Bikes, Ton Cars y Motos Roll
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/comercial/TNR-datos-para-el-analisis.xlsx
+++ b/comercial/TNR-datos-para-el-analisis.xlsx
@@ -947,7 +947,7 @@
       </c>
       <c r="J6" s="14" t="inlineStr">
         <is>
-          <t>A confirmar</t>
+          <t>Conforme (según Mateo)</t>
         </is>
       </c>
       <c r="K6" s="14" t="inlineStr">
@@ -968,7 +968,7 @@
       </c>
       <c r="O6" s="16" t="inlineStr">
         <is>
-          <t>A confirmar</t>
+          <t>Referido: la profe de Santi le dio una tarjeta a su pareja</t>
         </is>
       </c>
     </row>
@@ -1150,7 +1150,7 @@
       </c>
       <c r="J9" s="14" t="inlineStr">
         <is>
-          <t>A confirmar</t>
+          <t>Conformes (según Mateo). Mari, la que sabe, está muy contenta</t>
         </is>
       </c>
       <c r="K9" s="14" t="inlineStr">
@@ -1166,12 +1166,12 @@
       </c>
       <c r="N9" s="14" t="inlineStr">
         <is>
-          <t>E-commerce + branding 350.000 a 50.000 por semana (5ª semana). Queremos venderle redes.</t>
+          <t>Claudio es el dueño; la que decide lo digital es Mari. E-commerce + branding 350.000 a 50.000 por semana (5ª semana). Queremos venderle redes.</t>
         </is>
       </c>
       <c r="O9" s="16" t="inlineStr">
         <is>
-          <t>A confirmar</t>
+          <t>Prospección por WhatsApp</t>
         </is>
       </c>
     </row>
@@ -1215,7 +1215,7 @@
       </c>
       <c r="J10" s="14" t="inlineStr">
         <is>
-          <t>A confirmar</t>
+          <t>Conforme con la página (según Mateo)</t>
         </is>
       </c>
       <c r="K10" s="14" t="inlineStr">
@@ -1231,7 +1231,7 @@
       </c>
       <c r="N10" s="14" t="inlineStr">
         <is>
-          <t>Web 300.000 bruto; 30% al vendedor (el CRM guarda el neto: 210.000). Pagó 200.000, última cuota de 100.000 el 08/10. Panel nuevo a cobrar: 300.000.</t>
+          <t>Web 300.000 bruto; 30% al vendedor (el CRM guarda el neto). Pagó 200.000, última cuota de 100.000 el 08/10. Quiere el /admin (300.000) justamente para no pagar mensualidad.</t>
         </is>
       </c>
       <c r="O10" s="16" t="inlineStr">
@@ -1284,7 +1284,7 @@
       </c>
       <c r="J11" s="14" t="inlineStr">
         <is>
-          <t>A confirmar</t>
+          <t>Conforme con la web y con el mes gratis (según Mateo)</t>
         </is>
       </c>
       <c r="K11" s="14" t="inlineStr">

</xml_diff>

<commit_message>
Origen de Ciro, Kaiken, Ocampos y Thiago
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/comercial/TNR-datos-para-el-analisis.xlsx
+++ b/comercial/TNR-datos-para-el-analisis.xlsx
@@ -1037,7 +1037,7 @@
       </c>
       <c r="O7" s="16" t="inlineStr">
         <is>
-          <t>A confirmar</t>
+          <t>Prospección por mensajes</t>
         </is>
       </c>
     </row>
@@ -1508,7 +1508,7 @@
       </c>
       <c r="O14" s="16" t="inlineStr">
         <is>
-          <t>A confirmar</t>
+          <t>Alianza estratégica, después nos contrató</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
       </c>
       <c r="O16" s="16" t="inlineStr">
         <is>
-          <t>A confirmar</t>
+          <t>Cara a cara: charla en un Uber + tarjeta</t>
         </is>
       </c>
     </row>
@@ -1776,7 +1776,7 @@
       </c>
       <c r="O18" s="16" t="inlineStr">
         <is>
-          <t>A confirmar</t>
+          <t>Prospección por mensajes</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Lista de precios: piso en lo ya cobrado, redes por horas de grabacion
Webs y mensuales con el precio mas alto que un cliente ya pago; tienda,
branding y redes con la cuenta de horas y referencias de mercado. Reglas:
solo la demo es gratis, maximo 3 cuotas, ajuste trimestral anunciado.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/comercial/TNR-datos-para-el-analisis.xlsx
+++ b/comercial/TNR-datos-para-el-analisis.xlsx
@@ -13,6 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Facturacion" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobros" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Precios" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lista de precios" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -149,7 +150,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -188,6 +189,9 @@
     </xf>
     <xf numFmtId="3" fontId="13" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -5830,4 +5834,340 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Lista de precios desde el 19/09/2026 (clientes nuevos)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>El detalle y el porqué de cada número están en comercial/precios.md. Pesos, sin IVA. Ajuste cada 3 meses.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="24" t="inlineStr">
+        <is>
+          <t>Servicio</t>
+        </is>
+      </c>
+      <c r="B4" s="24" t="inlineStr">
+        <is>
+          <t>Precio ($)</t>
+        </is>
+      </c>
+      <c r="C4" s="24" t="inlineStr">
+        <is>
+          <t>Único o mensual</t>
+        </is>
+      </c>
+      <c r="D4" s="24" t="inlineStr">
+        <is>
+          <t>Qué incluye</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Web de una página</t>
+        </is>
+      </c>
+      <c r="B5" s="23" t="n">
+        <v>300000</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Único</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Secciones, WhatsApp, mapa, dominio</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Web + SEO local</t>
+        </is>
+      </c>
+      <c r="B6" s="23" t="n">
+        <v>350000</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Único</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Lo anterior + posicionamiento en la zona</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Web con blog</t>
+        </is>
+      </c>
+      <c r="B7" s="23" t="n">
+        <v>540000</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Único</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Varias páginas + blog</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Panel para autoadministrar (/admin)</t>
+        </is>
+      </c>
+      <c r="B8" s="23" t="n">
+        <v>300000</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Único</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Adicional a la web</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Tienda online</t>
+        </is>
+      </c>
+      <c r="B9" s="23" t="n">
+        <v>500000</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Único</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Hasta 30 productos cargados, carrito, pagos, envíos, panel</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Branding básico</t>
+        </is>
+      </c>
+      <c r="B10" s="23" t="n">
+        <v>150000</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Único</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Logo, paleta, tipografías, 5 aplicaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Identidad completa</t>
+        </is>
+      </c>
+      <c r="B11" s="23" t="n">
+        <v>350000</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Único</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Básico + charla de marca + manual + plantillas</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Mantenimiento web</t>
+        </is>
+      </c>
+      <c r="B12" s="23" t="n">
+        <v>100000</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Mensual</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Hosting y dominio, cambios, que ande</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Gestión de Google o Meta Ads</t>
+        </is>
+      </c>
+      <c r="B13" s="23" t="n">
+        <v>100000</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Mensual</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Más la inversión en anuncios, que paga el cliente</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Redes sin grabación</t>
+        </is>
+      </c>
+      <c r="B14" s="23" t="n">
+        <v>180000</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Mensual</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>15 piezas + estrategia + informe</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Redes con grabación</t>
+        </is>
+      </c>
+      <c r="B15" s="23" t="n">
+        <v>350000</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Mensual</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>15 contenidos con hasta 8 reels + estrategia + informe</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Reel extra dentro del plan</t>
+        </is>
+      </c>
+      <c r="B16" s="23" t="n">
+        <v>35000</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Mensual</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Arriba de los 8</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Reel suelto</t>
+        </is>
+      </c>
+      <c r="B17" s="23" t="n">
+        <v>60000</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Único</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Sin plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Demo de web</t>
+        </is>
+      </c>
+      <c r="B18" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Único</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Lo único gratis. Se muestra en llamada o en persona</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Ads: desde 150.000 o 15% de la inversion, con referencias de mercado
Los 100.000 salian de lo ya cobrado y quedaban debajo del piso del
mercado. Sube a 250-350 mil cuando haya casos de Meta con numeros.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/comercial/TNR-datos-para-el-analisis.xlsx
+++ b/comercial/TNR-datos-para-el-analisis.xlsx
@@ -6054,7 +6054,7 @@
         </is>
       </c>
       <c r="B13" s="23" t="n">
-        <v>100000</v>
+        <v>150000</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -6063,7 +6063,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Más la inversión en anuncios, que paga el cliente</t>
+          <t>Desde 150.000 o el 15% de la inversión, lo que sea mayor. La inversión la paga el cliente</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Todos los clientes reales autorizan: se saca el pendiente de todos lados
La columna de la hoja Clientes queda en Si para los 14, el prompt de
carruseles ya no pide preguntar y se borra el pendiente de Setup.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/comercial/TNR-datos-para-el-analisis.xlsx
+++ b/comercial/TNR-datos-para-el-analisis.xlsx
@@ -890,7 +890,11 @@
           <t>Real</t>
         </is>
       </c>
-      <c r="L5" s="11" t="inlineStr"/>
+      <c r="L5" s="11" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="M5" s="11" t="inlineStr">
         <is>
           <t>09/2026</t>
@@ -959,7 +963,11 @@
           <t>Real</t>
         </is>
       </c>
-      <c r="L6" s="14" t="inlineStr"/>
+      <c r="L6" s="14" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="M6" s="14" t="inlineStr">
         <is>
           <t>08/2026</t>
@@ -1028,7 +1036,11 @@
           <t>Real</t>
         </is>
       </c>
-      <c r="L7" s="14" t="inlineStr"/>
+      <c r="L7" s="14" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="M7" s="14" t="inlineStr">
         <is>
           <t>09/2026</t>
@@ -1093,7 +1105,11 @@
           <t>Real</t>
         </is>
       </c>
-      <c r="L8" s="14" t="inlineStr"/>
+      <c r="L8" s="14" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="M8" s="14" t="inlineStr">
         <is>
           <t>09/2026</t>
@@ -1162,7 +1178,11 @@
           <t>Real</t>
         </is>
       </c>
-      <c r="L9" s="14" t="inlineStr"/>
+      <c r="L9" s="14" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="M9" s="14" t="inlineStr">
         <is>
           <t>09/2026</t>
@@ -1227,7 +1247,11 @@
           <t>Real</t>
         </is>
       </c>
-      <c r="L10" s="14" t="inlineStr"/>
+      <c r="L10" s="14" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="M10" s="14" t="inlineStr">
         <is>
           <t>09/2026</t>
@@ -1296,7 +1320,11 @@
           <t>Real</t>
         </is>
       </c>
-      <c r="L11" s="14" t="inlineStr"/>
+      <c r="L11" s="14" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="M11" s="14" t="inlineStr">
         <is>
           <t>09/2026</t>
@@ -1365,7 +1393,11 @@
           <t>Real</t>
         </is>
       </c>
-      <c r="L12" s="14" t="inlineStr"/>
+      <c r="L12" s="14" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="M12" s="14" t="inlineStr">
         <is>
           <t>09/2026</t>
@@ -1434,7 +1466,11 @@
           <t>Real</t>
         </is>
       </c>
-      <c r="L13" s="14" t="inlineStr"/>
+      <c r="L13" s="14" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="M13" s="14" t="inlineStr">
         <is>
           <t>06/2026</t>
@@ -1499,7 +1535,11 @@
           <t>Real</t>
         </is>
       </c>
-      <c r="L14" s="14" t="inlineStr"/>
+      <c r="L14" s="14" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="M14" s="14" t="inlineStr">
         <is>
           <t>08/2026</t>
@@ -1568,7 +1608,11 @@
           <t>Real</t>
         </is>
       </c>
-      <c r="L15" s="14" t="inlineStr"/>
+      <c r="L15" s="14" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="M15" s="14" t="inlineStr">
         <is>
           <t>07/2026</t>
@@ -1637,7 +1681,11 @@
           <t>Real</t>
         </is>
       </c>
-      <c r="L16" s="14" t="inlineStr"/>
+      <c r="L16" s="14" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="M16" s="14" t="inlineStr">
         <is>
           <t>06/2026</t>
@@ -1706,7 +1754,11 @@
           <t>Real</t>
         </is>
       </c>
-      <c r="L17" s="14" t="inlineStr"/>
+      <c r="L17" s="14" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="M17" s="14" t="inlineStr">
         <is>
           <t>06/2026</t>
@@ -1767,7 +1819,11 @@
           <t>Real</t>
         </is>
       </c>
-      <c r="L18" s="14" t="inlineStr"/>
+      <c r="L18" s="14" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="M18" s="14" t="inlineStr">
         <is>
           <t>06/2026</t>

</xml_diff>